<commit_message>
Daily slate 2026-04-01 [auto]
</commit_message>
<xml_diff>
--- a/NBA/step8_nba1h_direction_clean.xlsx
+++ b/NBA/step8_nba1h_direction_clean.xlsx
@@ -1826,7 +1826,7 @@
       </c>
       <c r="BE6" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="BE7" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="BE12" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="BE16" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4134,7 @@
       </c>
       <c r="BE18" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="BE22" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5099,7 @@
       </c>
       <c r="BE23" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -6221,7 +6221,7 @@
       </c>
       <c r="BE29" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -7005,7 +7005,7 @@
       </c>
       <c r="BE33" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -7785,7 +7785,7 @@
       </c>
       <c r="BE37" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -13904,7 +13904,7 @@
       </c>
       <c r="BE72" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -14035,7 +14035,7 @@
       </c>
       <c r="BE73" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -14714,7 +14714,7 @@
       </c>
       <c r="BE78" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -15123,7 +15123,7 @@
       </c>
       <c r="BE81" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -16108,7 +16108,7 @@
       </c>
       <c r="BE88" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -16239,7 +16239,7 @@
       </c>
       <c r="BE89" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -17264,7 +17264,7 @@
       </c>
       <c r="BE96" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -17665,7 +17665,7 @@
       </c>
       <c r="BE99" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -19547,7 +19547,7 @@
       </c>
       <c r="BE4" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -19736,7 +19736,7 @@
       </c>
       <c r="BE5" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -20713,7 +20713,7 @@
       </c>
       <c r="BE10" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -21489,7 +21489,7 @@
       </c>
       <c r="BE14" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -22216,7 +22216,7 @@
       </c>
       <c r="BE3" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -22992,7 +22992,7 @@
       </c>
       <c r="BE7" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -23181,7 +23181,7 @@
       </c>
       <c r="BE8" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -24303,7 +24303,7 @@
       </c>
       <c r="BE14" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -25087,7 +25087,7 @@
       </c>
       <c r="BE18" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -25867,7 +25867,7 @@
       </c>
       <c r="BE22" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -31986,7 +31986,7 @@
       </c>
       <c r="BE57" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -32117,7 +32117,7 @@
       </c>
       <c r="BE58" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -32796,7 +32796,7 @@
       </c>
       <c r="BE63" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -33205,7 +33205,7 @@
       </c>
       <c r="BE66" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -34190,7 +34190,7 @@
       </c>
       <c r="BE73" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -34321,7 +34321,7 @@
       </c>
       <c r="BE74" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, fantasy: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -35346,7 +35346,7 @@
       </c>
       <c r="BE81" s="5" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pts: 1.06x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>
@@ -35747,7 +35747,7 @@
       </c>
       <c r="BE84" s="3" t="inlineStr">
         <is>
-          <t>PHI +16.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
+          <t>PHI +15.5 pt margin vs WSH, pra: 1.05x game script (fav; spread_risk 1.05, total_risk 1.02)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh sport pipeline outputs (MLB, NBA, NHL, Soccer) and update light UI theme
- Regenerate MLB/NBA/NHL/Soccer step outputs, caches, and direction workbooks
- Tune light theme to snow blue / blue-white surfaces (page shell, nav, index)
- Adjust run_daily.ps1 and ticket_eval_slate_latest.json

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/NBA/step8_nba1h_direction_clean.xlsx
+++ b/NBA/step8_nba1h_direction_clean.xlsx
@@ -13,10 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier D" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ALL'!$A$1:$BG$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tier B'!$A$1:$BG$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tier C'!$A$1:$BG$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Tier D'!$A$1:$BG$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ALL'!$A$1:$BJ$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tier B'!$A$1:$BJ$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tier C'!$A$1:$BJ$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Tier D'!$A$1:$BJ$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG90"/>
+  <dimension ref="A1:BJ90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -566,6 +566,9 @@
     <col width="12" customWidth="1" min="57" max="57"/>
     <col width="12" customWidth="1" min="58" max="58"/>
     <col width="12" customWidth="1" min="59" max="59"/>
+    <col width="12" customWidth="1" min="60" max="60"/>
+    <col width="12" customWidth="1" min="61" max="61"/>
+    <col width="12" customWidth="1" min="62" max="62"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -836,30 +839,45 @@
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
+          <t>H2H Over% (L5)</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>L5 vs Opp Hit%</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>Days Rest</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>Game Total</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>Spread</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Playoff Game</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>Game Script Mult</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>Game Script Note</t>
         </is>
@@ -1049,12 +1067,19 @@
       <c r="BC2" s="3" t="inlineStr"/>
       <c r="BD2" s="3" t="inlineStr"/>
       <c r="BE2" s="3" t="inlineStr"/>
-      <c r="BF2" s="3" t="inlineStr">
+      <c r="BF2" s="3" t="inlineStr"/>
+      <c r="BG2" s="3" t="inlineStr"/>
+      <c r="BH2" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI2" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG2" s="3" t="inlineStr">
+      <c r="BJ2" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -1260,12 +1285,19 @@
       <c r="BC3" s="5" t="inlineStr"/>
       <c r="BD3" s="5" t="inlineStr"/>
       <c r="BE3" s="5" t="inlineStr"/>
-      <c r="BF3" s="5" t="inlineStr">
+      <c r="BF3" s="5" t="inlineStr"/>
+      <c r="BG3" s="5" t="inlineStr"/>
+      <c r="BH3" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI3" s="5" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG3" s="5" t="inlineStr">
+      <c r="BJ3" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -1475,12 +1507,19 @@
       <c r="BC4" s="3" t="inlineStr"/>
       <c r="BD4" s="3" t="inlineStr"/>
       <c r="BE4" s="3" t="inlineStr"/>
-      <c r="BF4" s="3" t="inlineStr">
+      <c r="BF4" s="3" t="inlineStr"/>
+      <c r="BG4" s="3" t="inlineStr"/>
+      <c r="BH4" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI4" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG4" s="3" t="inlineStr">
+      <c r="BJ4" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -1666,12 +1705,19 @@
       <c r="BC5" s="5" t="inlineStr"/>
       <c r="BD5" s="5" t="inlineStr"/>
       <c r="BE5" s="5" t="inlineStr"/>
-      <c r="BF5" s="5" t="inlineStr">
+      <c r="BF5" s="5" t="inlineStr"/>
+      <c r="BG5" s="5" t="inlineStr"/>
+      <c r="BH5" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI5" s="5" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG5" s="5" t="inlineStr">
+      <c r="BJ5" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -1881,12 +1927,19 @@
       <c r="BC6" s="3" t="inlineStr"/>
       <c r="BD6" s="3" t="inlineStr"/>
       <c r="BE6" s="3" t="inlineStr"/>
-      <c r="BF6" s="3" t="inlineStr">
+      <c r="BF6" s="3" t="inlineStr"/>
+      <c r="BG6" s="3" t="inlineStr"/>
+      <c r="BH6" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI6" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG6" s="3" t="inlineStr">
+      <c r="BJ6" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -2080,12 +2133,19 @@
       <c r="BC7" s="5" t="inlineStr"/>
       <c r="BD7" s="5" t="inlineStr"/>
       <c r="BE7" s="5" t="inlineStr"/>
-      <c r="BF7" s="5" t="inlineStr">
+      <c r="BF7" s="5" t="inlineStr"/>
+      <c r="BG7" s="5" t="inlineStr"/>
+      <c r="BH7" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI7" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG7" s="5" t="inlineStr">
+      <c r="BJ7" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -2279,12 +2339,19 @@
       <c r="BC8" s="3" t="inlineStr"/>
       <c r="BD8" s="3" t="inlineStr"/>
       <c r="BE8" s="3" t="inlineStr"/>
-      <c r="BF8" s="3" t="inlineStr">
+      <c r="BF8" s="3" t="inlineStr"/>
+      <c r="BG8" s="3" t="inlineStr"/>
+      <c r="BH8" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI8" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG8" s="3" t="inlineStr">
+      <c r="BJ8" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -2490,12 +2557,19 @@
       <c r="BC9" s="5" t="inlineStr"/>
       <c r="BD9" s="5" t="inlineStr"/>
       <c r="BE9" s="5" t="inlineStr"/>
-      <c r="BF9" s="5" t="inlineStr">
+      <c r="BF9" s="5" t="inlineStr"/>
+      <c r="BG9" s="5" t="inlineStr"/>
+      <c r="BH9" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI9" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG9" s="5" t="inlineStr">
+      <c r="BJ9" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -2705,12 +2779,19 @@
       <c r="BC10" s="3" t="inlineStr"/>
       <c r="BD10" s="3" t="inlineStr"/>
       <c r="BE10" s="3" t="inlineStr"/>
-      <c r="BF10" s="3" t="inlineStr">
+      <c r="BF10" s="3" t="inlineStr"/>
+      <c r="BG10" s="3" t="inlineStr"/>
+      <c r="BH10" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI10" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG10" s="3" t="inlineStr">
+      <c r="BJ10" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -2920,12 +3001,19 @@
       <c r="BC11" s="5" t="inlineStr"/>
       <c r="BD11" s="5" t="inlineStr"/>
       <c r="BE11" s="5" t="inlineStr"/>
-      <c r="BF11" s="5" t="inlineStr">
+      <c r="BF11" s="5" t="inlineStr"/>
+      <c r="BG11" s="5" t="inlineStr"/>
+      <c r="BH11" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI11" s="5" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG11" s="5" t="inlineStr">
+      <c r="BJ11" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -3123,12 +3211,19 @@
       <c r="BC12" s="3" t="inlineStr"/>
       <c r="BD12" s="3" t="inlineStr"/>
       <c r="BE12" s="3" t="inlineStr"/>
-      <c r="BF12" s="3" t="inlineStr">
+      <c r="BF12" s="3" t="inlineStr"/>
+      <c r="BG12" s="3" t="inlineStr"/>
+      <c r="BH12" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI12" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG12" s="3" t="inlineStr">
+      <c r="BJ12" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -3338,12 +3433,19 @@
       <c r="BC13" s="5" t="inlineStr"/>
       <c r="BD13" s="5" t="inlineStr"/>
       <c r="BE13" s="5" t="inlineStr"/>
-      <c r="BF13" s="5" t="inlineStr">
+      <c r="BF13" s="5" t="inlineStr"/>
+      <c r="BG13" s="5" t="inlineStr"/>
+      <c r="BH13" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI13" s="5" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG13" s="5" t="inlineStr">
+      <c r="BJ13" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -3521,12 +3623,19 @@
       <c r="BC14" s="3" t="inlineStr"/>
       <c r="BD14" s="3" t="inlineStr"/>
       <c r="BE14" s="3" t="inlineStr"/>
-      <c r="BF14" s="3" t="inlineStr">
+      <c r="BF14" s="3" t="inlineStr"/>
+      <c r="BG14" s="3" t="inlineStr"/>
+      <c r="BH14" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI14" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG14" s="3" t="inlineStr">
+      <c r="BJ14" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -3728,12 +3837,19 @@
       <c r="BC15" s="5" t="inlineStr"/>
       <c r="BD15" s="5" t="inlineStr"/>
       <c r="BE15" s="5" t="inlineStr"/>
-      <c r="BF15" s="5" t="inlineStr">
+      <c r="BF15" s="5" t="inlineStr"/>
+      <c r="BG15" s="5" t="inlineStr"/>
+      <c r="BH15" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI15" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG15" s="5" t="inlineStr">
+      <c r="BJ15" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -3939,12 +4055,19 @@
       <c r="BC16" s="3" t="inlineStr"/>
       <c r="BD16" s="3" t="inlineStr"/>
       <c r="BE16" s="3" t="inlineStr"/>
-      <c r="BF16" s="3" t="inlineStr">
+      <c r="BF16" s="3" t="inlineStr"/>
+      <c r="BG16" s="3" t="inlineStr"/>
+      <c r="BH16" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI16" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG16" s="3" t="inlineStr">
+      <c r="BJ16" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -4154,12 +4277,19 @@
       <c r="BC17" s="5" t="inlineStr"/>
       <c r="BD17" s="5" t="inlineStr"/>
       <c r="BE17" s="5" t="inlineStr"/>
-      <c r="BF17" s="5" t="inlineStr">
+      <c r="BF17" s="5" t="inlineStr"/>
+      <c r="BG17" s="5" t="inlineStr"/>
+      <c r="BH17" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI17" s="5" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG17" s="5" t="inlineStr">
+      <c r="BJ17" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -4365,12 +4495,19 @@
       <c r="BC18" s="3" t="inlineStr"/>
       <c r="BD18" s="3" t="inlineStr"/>
       <c r="BE18" s="3" t="inlineStr"/>
-      <c r="BF18" s="3" t="inlineStr">
+      <c r="BF18" s="3" t="inlineStr"/>
+      <c r="BG18" s="3" t="inlineStr"/>
+      <c r="BH18" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI18" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG18" s="3" t="inlineStr">
+      <c r="BJ18" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -4560,12 +4697,19 @@
       <c r="BC19" s="5" t="inlineStr"/>
       <c r="BD19" s="5" t="inlineStr"/>
       <c r="BE19" s="5" t="inlineStr"/>
-      <c r="BF19" s="5" t="inlineStr">
+      <c r="BF19" s="5" t="inlineStr"/>
+      <c r="BG19" s="5" t="inlineStr"/>
+      <c r="BH19" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI19" s="5" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG19" s="5" t="inlineStr">
+      <c r="BJ19" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -4775,12 +4919,19 @@
       <c r="BC20" s="3" t="inlineStr"/>
       <c r="BD20" s="3" t="inlineStr"/>
       <c r="BE20" s="3" t="inlineStr"/>
-      <c r="BF20" s="3" t="inlineStr">
+      <c r="BF20" s="3" t="inlineStr"/>
+      <c r="BG20" s="3" t="inlineStr"/>
+      <c r="BH20" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI20" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG20" s="3" t="inlineStr">
+      <c r="BJ20" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -4990,12 +5141,19 @@
       <c r="BC21" s="5" t="inlineStr"/>
       <c r="BD21" s="5" t="inlineStr"/>
       <c r="BE21" s="5" t="inlineStr"/>
-      <c r="BF21" s="5" t="inlineStr">
+      <c r="BF21" s="5" t="inlineStr"/>
+      <c r="BG21" s="5" t="inlineStr"/>
+      <c r="BH21" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI21" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG21" s="5" t="inlineStr">
+      <c r="BJ21" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -5201,12 +5359,19 @@
       <c r="BC22" s="3" t="inlineStr"/>
       <c r="BD22" s="3" t="inlineStr"/>
       <c r="BE22" s="3" t="inlineStr"/>
-      <c r="BF22" s="3" t="inlineStr">
+      <c r="BF22" s="3" t="inlineStr"/>
+      <c r="BG22" s="3" t="inlineStr"/>
+      <c r="BH22" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI22" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG22" s="3" t="inlineStr">
+      <c r="BJ22" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -5408,12 +5573,19 @@
       <c r="BC23" s="5" t="inlineStr"/>
       <c r="BD23" s="5" t="inlineStr"/>
       <c r="BE23" s="5" t="inlineStr"/>
-      <c r="BF23" s="5" t="inlineStr">
+      <c r="BF23" s="5" t="inlineStr"/>
+      <c r="BG23" s="5" t="inlineStr"/>
+      <c r="BH23" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI23" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG23" s="5" t="inlineStr">
+      <c r="BJ23" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -5619,12 +5791,19 @@
       <c r="BC24" s="3" t="inlineStr"/>
       <c r="BD24" s="3" t="inlineStr"/>
       <c r="BE24" s="3" t="inlineStr"/>
-      <c r="BF24" s="3" t="inlineStr">
+      <c r="BF24" s="3" t="inlineStr"/>
+      <c r="BG24" s="3" t="inlineStr"/>
+      <c r="BH24" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI24" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG24" s="3" t="inlineStr">
+      <c r="BJ24" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -5826,12 +6005,19 @@
       <c r="BC25" s="5" t="inlineStr"/>
       <c r="BD25" s="5" t="inlineStr"/>
       <c r="BE25" s="5" t="inlineStr"/>
-      <c r="BF25" s="5" t="inlineStr">
+      <c r="BF25" s="5" t="inlineStr"/>
+      <c r="BG25" s="5" t="inlineStr"/>
+      <c r="BH25" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI25" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG25" s="5" t="inlineStr">
+      <c r="BJ25" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -6021,12 +6207,19 @@
       <c r="BC26" s="3" t="inlineStr"/>
       <c r="BD26" s="3" t="inlineStr"/>
       <c r="BE26" s="3" t="inlineStr"/>
-      <c r="BF26" s="3" t="inlineStr">
+      <c r="BF26" s="3" t="inlineStr"/>
+      <c r="BG26" s="3" t="inlineStr"/>
+      <c r="BH26" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI26" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG26" s="3" t="inlineStr">
+      <c r="BJ26" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -6236,12 +6429,19 @@
       <c r="BC27" s="5" t="inlineStr"/>
       <c r="BD27" s="5" t="inlineStr"/>
       <c r="BE27" s="5" t="inlineStr"/>
-      <c r="BF27" s="5" t="inlineStr">
+      <c r="BF27" s="5" t="inlineStr"/>
+      <c r="BG27" s="5" t="inlineStr"/>
+      <c r="BH27" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI27" s="5" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG27" s="5" t="inlineStr">
+      <c r="BJ27" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -6451,12 +6651,19 @@
       <c r="BC28" s="3" t="inlineStr"/>
       <c r="BD28" s="3" t="inlineStr"/>
       <c r="BE28" s="3" t="inlineStr"/>
-      <c r="BF28" s="3" t="inlineStr">
+      <c r="BF28" s="3" t="inlineStr"/>
+      <c r="BG28" s="3" t="inlineStr"/>
+      <c r="BH28" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI28" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG28" s="3" t="inlineStr">
+      <c r="BJ28" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -6662,12 +6869,19 @@
       <c r="BC29" s="5" t="inlineStr"/>
       <c r="BD29" s="5" t="inlineStr"/>
       <c r="BE29" s="5" t="inlineStr"/>
-      <c r="BF29" s="5" t="inlineStr">
+      <c r="BF29" s="5" t="inlineStr"/>
+      <c r="BG29" s="5" t="inlineStr"/>
+      <c r="BH29" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI29" s="5" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG29" s="5" t="inlineStr">
+      <c r="BJ29" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -6873,12 +7087,19 @@
       <c r="BC30" s="3" t="inlineStr"/>
       <c r="BD30" s="3" t="inlineStr"/>
       <c r="BE30" s="3" t="inlineStr"/>
-      <c r="BF30" s="3" t="inlineStr">
+      <c r="BF30" s="3" t="inlineStr"/>
+      <c r="BG30" s="3" t="inlineStr"/>
+      <c r="BH30" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI30" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG30" s="3" t="inlineStr">
+      <c r="BJ30" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -7088,12 +7309,19 @@
       <c r="BC31" s="5" t="inlineStr"/>
       <c r="BD31" s="5" t="inlineStr"/>
       <c r="BE31" s="5" t="inlineStr"/>
-      <c r="BF31" s="5" t="inlineStr">
+      <c r="BF31" s="5" t="inlineStr"/>
+      <c r="BG31" s="5" t="inlineStr"/>
+      <c r="BH31" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI31" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG31" s="5" t="inlineStr">
+      <c r="BJ31" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -7299,12 +7527,19 @@
       <c r="BC32" s="3" t="inlineStr"/>
       <c r="BD32" s="3" t="inlineStr"/>
       <c r="BE32" s="3" t="inlineStr"/>
-      <c r="BF32" s="3" t="inlineStr">
+      <c r="BF32" s="3" t="inlineStr"/>
+      <c r="BG32" s="3" t="inlineStr"/>
+      <c r="BH32" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI32" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG32" s="3" t="inlineStr">
+      <c r="BJ32" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -7506,12 +7741,19 @@
       <c r="BC33" s="5" t="inlineStr"/>
       <c r="BD33" s="5" t="inlineStr"/>
       <c r="BE33" s="5" t="inlineStr"/>
-      <c r="BF33" s="5" t="inlineStr">
+      <c r="BF33" s="5" t="inlineStr"/>
+      <c r="BG33" s="5" t="inlineStr"/>
+      <c r="BH33" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI33" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG33" s="5" t="inlineStr">
+      <c r="BJ33" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -7643,12 +7885,19 @@
       <c r="BC34" s="3" t="inlineStr"/>
       <c r="BD34" s="3" t="inlineStr"/>
       <c r="BE34" s="3" t="inlineStr"/>
-      <c r="BF34" s="3" t="inlineStr">
+      <c r="BF34" s="3" t="inlineStr"/>
+      <c r="BG34" s="3" t="inlineStr"/>
+      <c r="BH34" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI34" s="3" t="inlineStr">
         <is>
           <t>1.016</t>
         </is>
       </c>
-      <c r="BG34" s="3" t="inlineStr">
+      <c r="BJ34" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, 3ptmade: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -7780,12 +8029,19 @@
       <c r="BC35" s="5" t="inlineStr"/>
       <c r="BD35" s="5" t="inlineStr"/>
       <c r="BE35" s="5" t="inlineStr"/>
-      <c r="BF35" s="5" t="inlineStr">
+      <c r="BF35" s="5" t="inlineStr"/>
+      <c r="BG35" s="5" t="inlineStr"/>
+      <c r="BH35" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI35" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG35" s="5" t="inlineStr">
+      <c r="BJ35" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -7917,12 +8173,19 @@
       <c r="BC36" s="3" t="inlineStr"/>
       <c r="BD36" s="3" t="inlineStr"/>
       <c r="BE36" s="3" t="inlineStr"/>
-      <c r="BF36" s="3" t="inlineStr">
+      <c r="BF36" s="3" t="inlineStr"/>
+      <c r="BG36" s="3" t="inlineStr"/>
+      <c r="BH36" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI36" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG36" s="3" t="inlineStr">
+      <c r="BJ36" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -8054,12 +8317,19 @@
       <c r="BC37" s="5" t="inlineStr"/>
       <c r="BD37" s="5" t="inlineStr"/>
       <c r="BE37" s="5" t="inlineStr"/>
-      <c r="BF37" s="5" t="inlineStr">
+      <c r="BF37" s="5" t="inlineStr"/>
+      <c r="BG37" s="5" t="inlineStr"/>
+      <c r="BH37" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI37" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG37" s="5" t="inlineStr">
+      <c r="BJ37" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -8191,12 +8461,19 @@
       <c r="BC38" s="3" t="inlineStr"/>
       <c r="BD38" s="3" t="inlineStr"/>
       <c r="BE38" s="3" t="inlineStr"/>
-      <c r="BF38" s="3" t="inlineStr">
+      <c r="BF38" s="3" t="inlineStr"/>
+      <c r="BG38" s="3" t="inlineStr"/>
+      <c r="BH38" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI38" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG38" s="3" t="inlineStr">
+      <c r="BJ38" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -8328,12 +8605,19 @@
       <c r="BC39" s="5" t="inlineStr"/>
       <c r="BD39" s="5" t="inlineStr"/>
       <c r="BE39" s="5" t="inlineStr"/>
-      <c r="BF39" s="5" t="inlineStr">
+      <c r="BF39" s="5" t="inlineStr"/>
+      <c r="BG39" s="5" t="inlineStr"/>
+      <c r="BH39" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI39" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG39" s="5" t="inlineStr">
+      <c r="BJ39" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -8465,12 +8749,19 @@
       <c r="BC40" s="3" t="inlineStr"/>
       <c r="BD40" s="3" t="inlineStr"/>
       <c r="BE40" s="3" t="inlineStr"/>
-      <c r="BF40" s="3" t="inlineStr">
+      <c r="BF40" s="3" t="inlineStr"/>
+      <c r="BG40" s="3" t="inlineStr"/>
+      <c r="BH40" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI40" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG40" s="3" t="inlineStr">
+      <c r="BJ40" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -8602,12 +8893,19 @@
       <c r="BC41" s="5" t="inlineStr"/>
       <c r="BD41" s="5" t="inlineStr"/>
       <c r="BE41" s="5" t="inlineStr"/>
-      <c r="BF41" s="5" t="inlineStr">
+      <c r="BF41" s="5" t="inlineStr"/>
+      <c r="BG41" s="5" t="inlineStr"/>
+      <c r="BH41" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI41" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG41" s="5" t="inlineStr">
+      <c r="BJ41" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -8739,12 +9037,19 @@
       <c r="BC42" s="3" t="inlineStr"/>
       <c r="BD42" s="3" t="inlineStr"/>
       <c r="BE42" s="3" t="inlineStr"/>
-      <c r="BF42" s="3" t="inlineStr">
+      <c r="BF42" s="3" t="inlineStr"/>
+      <c r="BG42" s="3" t="inlineStr"/>
+      <c r="BH42" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI42" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG42" s="3" t="inlineStr">
+      <c r="BJ42" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -8876,12 +9181,19 @@
       <c r="BC43" s="5" t="inlineStr"/>
       <c r="BD43" s="5" t="inlineStr"/>
       <c r="BE43" s="5" t="inlineStr"/>
-      <c r="BF43" s="5" t="inlineStr">
+      <c r="BF43" s="5" t="inlineStr"/>
+      <c r="BG43" s="5" t="inlineStr"/>
+      <c r="BH43" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI43" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG43" s="5" t="inlineStr">
+      <c r="BJ43" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -9013,12 +9325,19 @@
       <c r="BC44" s="3" t="inlineStr"/>
       <c r="BD44" s="3" t="inlineStr"/>
       <c r="BE44" s="3" t="inlineStr"/>
-      <c r="BF44" s="3" t="inlineStr">
+      <c r="BF44" s="3" t="inlineStr"/>
+      <c r="BG44" s="3" t="inlineStr"/>
+      <c r="BH44" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI44" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG44" s="3" t="inlineStr">
+      <c r="BJ44" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -9210,12 +9529,19 @@
       <c r="BC45" s="5" t="inlineStr"/>
       <c r="BD45" s="5" t="inlineStr"/>
       <c r="BE45" s="5" t="inlineStr"/>
-      <c r="BF45" s="5" t="inlineStr">
+      <c r="BF45" s="5" t="inlineStr"/>
+      <c r="BG45" s="5" t="inlineStr"/>
+      <c r="BH45" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI45" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG45" s="5" t="inlineStr">
+      <c r="BJ45" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -9347,12 +9673,19 @@
       <c r="BC46" s="3" t="inlineStr"/>
       <c r="BD46" s="3" t="inlineStr"/>
       <c r="BE46" s="3" t="inlineStr"/>
-      <c r="BF46" s="3" t="inlineStr">
+      <c r="BF46" s="3" t="inlineStr"/>
+      <c r="BG46" s="3" t="inlineStr"/>
+      <c r="BH46" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI46" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG46" s="3" t="inlineStr">
+      <c r="BJ46" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -9560,12 +9893,19 @@
       <c r="BC47" s="5" t="inlineStr"/>
       <c r="BD47" s="5" t="inlineStr"/>
       <c r="BE47" s="5" t="inlineStr"/>
-      <c r="BF47" s="5" t="inlineStr">
+      <c r="BF47" s="5" t="inlineStr"/>
+      <c r="BG47" s="5" t="inlineStr"/>
+      <c r="BH47" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI47" s="5" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG47" s="5" t="inlineStr">
+      <c r="BJ47" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -9697,12 +10037,19 @@
       <c r="BC48" s="3" t="inlineStr"/>
       <c r="BD48" s="3" t="inlineStr"/>
       <c r="BE48" s="3" t="inlineStr"/>
-      <c r="BF48" s="3" t="inlineStr">
+      <c r="BF48" s="3" t="inlineStr"/>
+      <c r="BG48" s="3" t="inlineStr"/>
+      <c r="BH48" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI48" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG48" s="3" t="inlineStr">
+      <c r="BJ48" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -9834,12 +10181,19 @@
       <c r="BC49" s="5" t="inlineStr"/>
       <c r="BD49" s="5" t="inlineStr"/>
       <c r="BE49" s="5" t="inlineStr"/>
-      <c r="BF49" s="5" t="inlineStr">
+      <c r="BF49" s="5" t="inlineStr"/>
+      <c r="BG49" s="5" t="inlineStr"/>
+      <c r="BH49" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI49" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG49" s="5" t="inlineStr">
+      <c r="BJ49" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -10035,12 +10389,19 @@
       <c r="BC50" s="3" t="inlineStr"/>
       <c r="BD50" s="3" t="inlineStr"/>
       <c r="BE50" s="3" t="inlineStr"/>
-      <c r="BF50" s="3" t="inlineStr">
+      <c r="BF50" s="3" t="inlineStr"/>
+      <c r="BG50" s="3" t="inlineStr"/>
+      <c r="BH50" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI50" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG50" s="3" t="inlineStr">
+      <c r="BJ50" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -10172,12 +10533,19 @@
       <c r="BC51" s="5" t="inlineStr"/>
       <c r="BD51" s="5" t="inlineStr"/>
       <c r="BE51" s="5" t="inlineStr"/>
-      <c r="BF51" s="5" t="inlineStr">
+      <c r="BF51" s="5" t="inlineStr"/>
+      <c r="BG51" s="5" t="inlineStr"/>
+      <c r="BH51" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI51" s="5" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG51" s="5" t="inlineStr">
+      <c r="BJ51" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -10309,12 +10677,19 @@
       <c r="BC52" s="3" t="inlineStr"/>
       <c r="BD52" s="3" t="inlineStr"/>
       <c r="BE52" s="3" t="inlineStr"/>
-      <c r="BF52" s="3" t="inlineStr">
+      <c r="BF52" s="3" t="inlineStr"/>
+      <c r="BG52" s="3" t="inlineStr"/>
+      <c r="BH52" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI52" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG52" s="3" t="inlineStr">
+      <c r="BJ52" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -10446,12 +10821,19 @@
       <c r="BC53" s="5" t="inlineStr"/>
       <c r="BD53" s="5" t="inlineStr"/>
       <c r="BE53" s="5" t="inlineStr"/>
-      <c r="BF53" s="5" t="inlineStr">
+      <c r="BF53" s="5" t="inlineStr"/>
+      <c r="BG53" s="5" t="inlineStr"/>
+      <c r="BH53" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI53" s="5" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG53" s="5" t="inlineStr">
+      <c r="BJ53" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -10583,12 +10965,19 @@
       <c r="BC54" s="3" t="inlineStr"/>
       <c r="BD54" s="3" t="inlineStr"/>
       <c r="BE54" s="3" t="inlineStr"/>
-      <c r="BF54" s="3" t="inlineStr">
+      <c r="BF54" s="3" t="inlineStr"/>
+      <c r="BG54" s="3" t="inlineStr"/>
+      <c r="BH54" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI54" s="3" t="inlineStr">
         <is>
           <t>1.016</t>
         </is>
       </c>
-      <c r="BG54" s="3" t="inlineStr">
+      <c r="BJ54" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, 3ptmade: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -10720,12 +11109,19 @@
       <c r="BC55" s="5" t="inlineStr"/>
       <c r="BD55" s="5" t="inlineStr"/>
       <c r="BE55" s="5" t="inlineStr"/>
-      <c r="BF55" s="5" t="inlineStr">
+      <c r="BF55" s="5" t="inlineStr"/>
+      <c r="BG55" s="5" t="inlineStr"/>
+      <c r="BH55" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI55" s="5" t="inlineStr">
         <is>
           <t>1.016</t>
         </is>
       </c>
-      <c r="BG55" s="5" t="inlineStr">
+      <c r="BJ55" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, 3ptmade: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -10857,12 +11253,19 @@
       <c r="BC56" s="3" t="inlineStr"/>
       <c r="BD56" s="3" t="inlineStr"/>
       <c r="BE56" s="3" t="inlineStr"/>
-      <c r="BF56" s="3" t="inlineStr">
+      <c r="BF56" s="3" t="inlineStr"/>
+      <c r="BG56" s="3" t="inlineStr"/>
+      <c r="BH56" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI56" s="3" t="inlineStr">
         <is>
           <t>1.016</t>
         </is>
       </c>
-      <c r="BG56" s="3" t="inlineStr">
+      <c r="BJ56" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, 3ptmade: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -10994,12 +11397,19 @@
       <c r="BC57" s="5" t="inlineStr"/>
       <c r="BD57" s="5" t="inlineStr"/>
       <c r="BE57" s="5" t="inlineStr"/>
-      <c r="BF57" s="5" t="inlineStr">
+      <c r="BF57" s="5" t="inlineStr"/>
+      <c r="BG57" s="5" t="inlineStr"/>
+      <c r="BH57" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI57" s="5" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG57" s="5" t="inlineStr">
+      <c r="BJ57" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -11131,12 +11541,19 @@
       <c r="BC58" s="3" t="inlineStr"/>
       <c r="BD58" s="3" t="inlineStr"/>
       <c r="BE58" s="3" t="inlineStr"/>
-      <c r="BF58" s="3" t="inlineStr">
+      <c r="BF58" s="3" t="inlineStr"/>
+      <c r="BG58" s="3" t="inlineStr"/>
+      <c r="BH58" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI58" s="3" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG58" s="3" t="inlineStr">
+      <c r="BJ58" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -11268,12 +11685,19 @@
       <c r="BC59" s="5" t="inlineStr"/>
       <c r="BD59" s="5" t="inlineStr"/>
       <c r="BE59" s="5" t="inlineStr"/>
-      <c r="BF59" s="5" t="inlineStr">
+      <c r="BF59" s="5" t="inlineStr"/>
+      <c r="BG59" s="5" t="inlineStr"/>
+      <c r="BH59" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI59" s="5" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG59" s="5" t="inlineStr">
+      <c r="BJ59" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -11405,12 +11829,19 @@
       <c r="BC60" s="3" t="inlineStr"/>
       <c r="BD60" s="3" t="inlineStr"/>
       <c r="BE60" s="3" t="inlineStr"/>
-      <c r="BF60" s="3" t="inlineStr">
+      <c r="BF60" s="3" t="inlineStr"/>
+      <c r="BG60" s="3" t="inlineStr"/>
+      <c r="BH60" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI60" s="3" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG60" s="3" t="inlineStr">
+      <c r="BJ60" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -11542,12 +11973,19 @@
       <c r="BC61" s="5" t="inlineStr"/>
       <c r="BD61" s="5" t="inlineStr"/>
       <c r="BE61" s="5" t="inlineStr"/>
-      <c r="BF61" s="5" t="inlineStr">
+      <c r="BF61" s="5" t="inlineStr"/>
+      <c r="BG61" s="5" t="inlineStr"/>
+      <c r="BH61" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI61" s="5" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG61" s="5" t="inlineStr">
+      <c r="BJ61" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -11679,12 +12117,19 @@
       <c r="BC62" s="3" t="inlineStr"/>
       <c r="BD62" s="3" t="inlineStr"/>
       <c r="BE62" s="3" t="inlineStr"/>
-      <c r="BF62" s="3" t="inlineStr">
+      <c r="BF62" s="3" t="inlineStr"/>
+      <c r="BG62" s="3" t="inlineStr"/>
+      <c r="BH62" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI62" s="3" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG62" s="3" t="inlineStr">
+      <c r="BJ62" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -11816,12 +12261,19 @@
       <c r="BC63" s="5" t="inlineStr"/>
       <c r="BD63" s="5" t="inlineStr"/>
       <c r="BE63" s="5" t="inlineStr"/>
-      <c r="BF63" s="5" t="inlineStr">
+      <c r="BF63" s="5" t="inlineStr"/>
+      <c r="BG63" s="5" t="inlineStr"/>
+      <c r="BH63" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI63" s="5" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG63" s="5" t="inlineStr">
+      <c r="BJ63" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -11953,12 +12405,19 @@
       <c r="BC64" s="3" t="inlineStr"/>
       <c r="BD64" s="3" t="inlineStr"/>
       <c r="BE64" s="3" t="inlineStr"/>
-      <c r="BF64" s="3" t="inlineStr">
+      <c r="BF64" s="3" t="inlineStr"/>
+      <c r="BG64" s="3" t="inlineStr"/>
+      <c r="BH64" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI64" s="3" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG64" s="3" t="inlineStr">
+      <c r="BJ64" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -12090,12 +12549,19 @@
       <c r="BC65" s="5" t="inlineStr"/>
       <c r="BD65" s="5" t="inlineStr"/>
       <c r="BE65" s="5" t="inlineStr"/>
-      <c r="BF65" s="5" t="inlineStr">
+      <c r="BF65" s="5" t="inlineStr"/>
+      <c r="BG65" s="5" t="inlineStr"/>
+      <c r="BH65" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI65" s="5" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG65" s="5" t="inlineStr">
+      <c r="BJ65" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -12227,12 +12693,19 @@
       <c r="BC66" s="3" t="inlineStr"/>
       <c r="BD66" s="3" t="inlineStr"/>
       <c r="BE66" s="3" t="inlineStr"/>
-      <c r="BF66" s="3" t="inlineStr">
+      <c r="BF66" s="3" t="inlineStr"/>
+      <c r="BG66" s="3" t="inlineStr"/>
+      <c r="BH66" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI66" s="3" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG66" s="3" t="inlineStr">
+      <c r="BJ66" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -12364,12 +12837,19 @@
       <c r="BC67" s="5" t="inlineStr"/>
       <c r="BD67" s="5" t="inlineStr"/>
       <c r="BE67" s="5" t="inlineStr"/>
-      <c r="BF67" s="5" t="inlineStr">
+      <c r="BF67" s="5" t="inlineStr"/>
+      <c r="BG67" s="5" t="inlineStr"/>
+      <c r="BH67" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI67" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG67" s="5" t="inlineStr">
+      <c r="BJ67" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -12501,12 +12981,19 @@
       <c r="BC68" s="3" t="inlineStr"/>
       <c r="BD68" s="3" t="inlineStr"/>
       <c r="BE68" s="3" t="inlineStr"/>
-      <c r="BF68" s="3" t="inlineStr">
+      <c r="BF68" s="3" t="inlineStr"/>
+      <c r="BG68" s="3" t="inlineStr"/>
+      <c r="BH68" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI68" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG68" s="3" t="inlineStr">
+      <c r="BJ68" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -12638,12 +13125,19 @@
       <c r="BC69" s="5" t="inlineStr"/>
       <c r="BD69" s="5" t="inlineStr"/>
       <c r="BE69" s="5" t="inlineStr"/>
-      <c r="BF69" s="5" t="inlineStr">
+      <c r="BF69" s="5" t="inlineStr"/>
+      <c r="BG69" s="5" t="inlineStr"/>
+      <c r="BH69" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI69" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG69" s="5" t="inlineStr">
+      <c r="BJ69" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -12775,12 +13269,19 @@
       <c r="BC70" s="3" t="inlineStr"/>
       <c r="BD70" s="3" t="inlineStr"/>
       <c r="BE70" s="3" t="inlineStr"/>
-      <c r="BF70" s="3" t="inlineStr">
+      <c r="BF70" s="3" t="inlineStr"/>
+      <c r="BG70" s="3" t="inlineStr"/>
+      <c r="BH70" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI70" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG70" s="3" t="inlineStr">
+      <c r="BJ70" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -12912,12 +13413,19 @@
       <c r="BC71" s="5" t="inlineStr"/>
       <c r="BD71" s="5" t="inlineStr"/>
       <c r="BE71" s="5" t="inlineStr"/>
-      <c r="BF71" s="5" t="inlineStr">
+      <c r="BF71" s="5" t="inlineStr"/>
+      <c r="BG71" s="5" t="inlineStr"/>
+      <c r="BH71" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI71" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG71" s="5" t="inlineStr">
+      <c r="BJ71" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -13049,12 +13557,19 @@
       <c r="BC72" s="3" t="inlineStr"/>
       <c r="BD72" s="3" t="inlineStr"/>
       <c r="BE72" s="3" t="inlineStr"/>
-      <c r="BF72" s="3" t="inlineStr">
+      <c r="BF72" s="3" t="inlineStr"/>
+      <c r="BG72" s="3" t="inlineStr"/>
+      <c r="BH72" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI72" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG72" s="3" t="inlineStr">
+      <c r="BJ72" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -13186,12 +13701,19 @@
       <c r="BC73" s="5" t="inlineStr"/>
       <c r="BD73" s="5" t="inlineStr"/>
       <c r="BE73" s="5" t="inlineStr"/>
-      <c r="BF73" s="5" t="inlineStr">
+      <c r="BF73" s="5" t="inlineStr"/>
+      <c r="BG73" s="5" t="inlineStr"/>
+      <c r="BH73" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI73" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG73" s="5" t="inlineStr">
+      <c r="BJ73" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -13323,12 +13845,19 @@
       <c r="BC74" s="3" t="inlineStr"/>
       <c r="BD74" s="3" t="inlineStr"/>
       <c r="BE74" s="3" t="inlineStr"/>
-      <c r="BF74" s="3" t="inlineStr">
+      <c r="BF74" s="3" t="inlineStr"/>
+      <c r="BG74" s="3" t="inlineStr"/>
+      <c r="BH74" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI74" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG74" s="3" t="inlineStr">
+      <c r="BJ74" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -13460,12 +13989,19 @@
       <c r="BC75" s="5" t="inlineStr"/>
       <c r="BD75" s="5" t="inlineStr"/>
       <c r="BE75" s="5" t="inlineStr"/>
-      <c r="BF75" s="5" t="inlineStr">
+      <c r="BF75" s="5" t="inlineStr"/>
+      <c r="BG75" s="5" t="inlineStr"/>
+      <c r="BH75" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI75" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG75" s="5" t="inlineStr">
+      <c r="BJ75" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -13597,12 +14133,19 @@
       <c r="BC76" s="3" t="inlineStr"/>
       <c r="BD76" s="3" t="inlineStr"/>
       <c r="BE76" s="3" t="inlineStr"/>
-      <c r="BF76" s="3" t="inlineStr">
+      <c r="BF76" s="3" t="inlineStr"/>
+      <c r="BG76" s="3" t="inlineStr"/>
+      <c r="BH76" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI76" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG76" s="3" t="inlineStr">
+      <c r="BJ76" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -13734,12 +14277,19 @@
       <c r="BC77" s="5" t="inlineStr"/>
       <c r="BD77" s="5" t="inlineStr"/>
       <c r="BE77" s="5" t="inlineStr"/>
-      <c r="BF77" s="5" t="inlineStr">
+      <c r="BF77" s="5" t="inlineStr"/>
+      <c r="BG77" s="5" t="inlineStr"/>
+      <c r="BH77" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI77" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG77" s="5" t="inlineStr">
+      <c r="BJ77" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -13871,12 +14421,19 @@
       <c r="BC78" s="3" t="inlineStr"/>
       <c r="BD78" s="3" t="inlineStr"/>
       <c r="BE78" s="3" t="inlineStr"/>
-      <c r="BF78" s="3" t="inlineStr">
+      <c r="BF78" s="3" t="inlineStr"/>
+      <c r="BG78" s="3" t="inlineStr"/>
+      <c r="BH78" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI78" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG78" s="3" t="inlineStr">
+      <c r="BJ78" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -14056,12 +14613,19 @@
       <c r="BC79" s="5" t="inlineStr"/>
       <c r="BD79" s="5" t="inlineStr"/>
       <c r="BE79" s="5" t="inlineStr"/>
-      <c r="BF79" s="5" t="inlineStr">
+      <c r="BF79" s="5" t="inlineStr"/>
+      <c r="BG79" s="5" t="inlineStr"/>
+      <c r="BH79" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI79" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG79" s="5" t="inlineStr">
+      <c r="BJ79" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -14193,12 +14757,19 @@
       <c r="BC80" s="3" t="inlineStr"/>
       <c r="BD80" s="3" t="inlineStr"/>
       <c r="BE80" s="3" t="inlineStr"/>
-      <c r="BF80" s="3" t="inlineStr">
+      <c r="BF80" s="3" t="inlineStr"/>
+      <c r="BG80" s="3" t="inlineStr"/>
+      <c r="BH80" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI80" s="3" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG80" s="3" t="inlineStr">
+      <c r="BJ80" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -14330,12 +14901,19 @@
       <c r="BC81" s="5" t="inlineStr"/>
       <c r="BD81" s="5" t="inlineStr"/>
       <c r="BE81" s="5" t="inlineStr"/>
-      <c r="BF81" s="5" t="inlineStr">
+      <c r="BF81" s="5" t="inlineStr"/>
+      <c r="BG81" s="5" t="inlineStr"/>
+      <c r="BH81" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI81" s="5" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG81" s="5" t="inlineStr">
+      <c r="BJ81" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -14467,12 +15045,19 @@
       <c r="BC82" s="3" t="inlineStr"/>
       <c r="BD82" s="3" t="inlineStr"/>
       <c r="BE82" s="3" t="inlineStr"/>
-      <c r="BF82" s="3" t="inlineStr">
+      <c r="BF82" s="3" t="inlineStr"/>
+      <c r="BG82" s="3" t="inlineStr"/>
+      <c r="BH82" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI82" s="3" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG82" s="3" t="inlineStr">
+      <c r="BJ82" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -14604,12 +15189,19 @@
       <c r="BC83" s="5" t="inlineStr"/>
       <c r="BD83" s="5" t="inlineStr"/>
       <c r="BE83" s="5" t="inlineStr"/>
-      <c r="BF83" s="5" t="inlineStr">
+      <c r="BF83" s="5" t="inlineStr"/>
+      <c r="BG83" s="5" t="inlineStr"/>
+      <c r="BH83" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI83" s="5" t="inlineStr">
         <is>
           <t>1.016</t>
         </is>
       </c>
-      <c r="BG83" s="5" t="inlineStr">
+      <c r="BJ83" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, 3ptmade: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -14741,12 +15333,19 @@
       <c r="BC84" s="3" t="inlineStr"/>
       <c r="BD84" s="3" t="inlineStr"/>
       <c r="BE84" s="3" t="inlineStr"/>
-      <c r="BF84" s="3" t="inlineStr">
+      <c r="BF84" s="3" t="inlineStr"/>
+      <c r="BG84" s="3" t="inlineStr"/>
+      <c r="BH84" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI84" s="3" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG84" s="3" t="inlineStr">
+      <c r="BJ84" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -14878,12 +15477,19 @@
       <c r="BC85" s="5" t="inlineStr"/>
       <c r="BD85" s="5" t="inlineStr"/>
       <c r="BE85" s="5" t="inlineStr"/>
-      <c r="BF85" s="5" t="inlineStr">
+      <c r="BF85" s="5" t="inlineStr"/>
+      <c r="BG85" s="5" t="inlineStr"/>
+      <c r="BH85" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI85" s="5" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG85" s="5" t="inlineStr">
+      <c r="BJ85" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -15015,12 +15621,19 @@
       <c r="BC86" s="3" t="inlineStr"/>
       <c r="BD86" s="3" t="inlineStr"/>
       <c r="BE86" s="3" t="inlineStr"/>
-      <c r="BF86" s="3" t="inlineStr">
+      <c r="BF86" s="3" t="inlineStr"/>
+      <c r="BG86" s="3" t="inlineStr"/>
+      <c r="BH86" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI86" s="3" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG86" s="3" t="inlineStr">
+      <c r="BJ86" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -15152,12 +15765,19 @@
       <c r="BC87" s="5" t="inlineStr"/>
       <c r="BD87" s="5" t="inlineStr"/>
       <c r="BE87" s="5" t="inlineStr"/>
-      <c r="BF87" s="5" t="inlineStr">
+      <c r="BF87" s="5" t="inlineStr"/>
+      <c r="BG87" s="5" t="inlineStr"/>
+      <c r="BH87" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI87" s="5" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG87" s="5" t="inlineStr">
+      <c r="BJ87" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -15289,12 +15909,19 @@
       <c r="BC88" s="3" t="inlineStr"/>
       <c r="BD88" s="3" t="inlineStr"/>
       <c r="BE88" s="3" t="inlineStr"/>
-      <c r="BF88" s="3" t="inlineStr">
+      <c r="BF88" s="3" t="inlineStr"/>
+      <c r="BG88" s="3" t="inlineStr"/>
+      <c r="BH88" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI88" s="3" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG88" s="3" t="inlineStr">
+      <c r="BJ88" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -15426,12 +16053,19 @@
       <c r="BC89" s="5" t="inlineStr"/>
       <c r="BD89" s="5" t="inlineStr"/>
       <c r="BE89" s="5" t="inlineStr"/>
-      <c r="BF89" s="5" t="inlineStr">
+      <c r="BF89" s="5" t="inlineStr"/>
+      <c r="BG89" s="5" t="inlineStr"/>
+      <c r="BH89" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI89" s="5" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG89" s="5" t="inlineStr">
+      <c r="BJ89" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -15563,19 +16197,26 @@
       <c r="BC90" s="3" t="inlineStr"/>
       <c r="BD90" s="3" t="inlineStr"/>
       <c r="BE90" s="3" t="inlineStr"/>
-      <c r="BF90" s="3" t="inlineStr">
+      <c r="BF90" s="3" t="inlineStr"/>
+      <c r="BG90" s="3" t="inlineStr"/>
+      <c r="BH90" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI90" s="3" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG90" s="3" t="inlineStr">
+      <c r="BJ90" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BG1"/>
+  <autoFilter ref="A1:BJ1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15586,7 +16227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG4"/>
+  <dimension ref="A1:BJ4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -15648,6 +16289,9 @@
     <col width="12" customWidth="1" min="57" max="57"/>
     <col width="12" customWidth="1" min="58" max="58"/>
     <col width="12" customWidth="1" min="59" max="59"/>
+    <col width="12" customWidth="1" min="60" max="60"/>
+    <col width="12" customWidth="1" min="61" max="61"/>
+    <col width="12" customWidth="1" min="62" max="62"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -15918,30 +16562,45 @@
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
+          <t>H2H Over% (L5)</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>L5 vs Opp Hit%</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>Days Rest</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>Game Total</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>Spread</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Playoff Game</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>Game Script Mult</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>Game Script Note</t>
         </is>
@@ -16131,12 +16790,19 @@
       <c r="BC2" s="3" t="inlineStr"/>
       <c r="BD2" s="3" t="inlineStr"/>
       <c r="BE2" s="3" t="inlineStr"/>
-      <c r="BF2" s="3" t="inlineStr">
+      <c r="BF2" s="3" t="inlineStr"/>
+      <c r="BG2" s="3" t="inlineStr"/>
+      <c r="BH2" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI2" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG2" s="3" t="inlineStr">
+      <c r="BJ2" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -16342,12 +17008,19 @@
       <c r="BC3" s="5" t="inlineStr"/>
       <c r="BD3" s="5" t="inlineStr"/>
       <c r="BE3" s="5" t="inlineStr"/>
-      <c r="BF3" s="5" t="inlineStr">
+      <c r="BF3" s="5" t="inlineStr"/>
+      <c r="BG3" s="5" t="inlineStr"/>
+      <c r="BH3" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI3" s="5" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG3" s="5" t="inlineStr">
+      <c r="BJ3" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -16557,19 +17230,26 @@
       <c r="BC4" s="3" t="inlineStr"/>
       <c r="BD4" s="3" t="inlineStr"/>
       <c r="BE4" s="3" t="inlineStr"/>
-      <c r="BF4" s="3" t="inlineStr">
+      <c r="BF4" s="3" t="inlineStr"/>
+      <c r="BG4" s="3" t="inlineStr"/>
+      <c r="BH4" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI4" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG4" s="3" t="inlineStr">
+      <c r="BJ4" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BG1"/>
+  <autoFilter ref="A1:BJ1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16580,7 +17260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG11"/>
+  <dimension ref="A1:BJ11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16642,6 +17322,9 @@
     <col width="12" customWidth="1" min="57" max="57"/>
     <col width="12" customWidth="1" min="58" max="58"/>
     <col width="12" customWidth="1" min="59" max="59"/>
+    <col width="12" customWidth="1" min="60" max="60"/>
+    <col width="12" customWidth="1" min="61" max="61"/>
+    <col width="12" customWidth="1" min="62" max="62"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -16912,30 +17595,45 @@
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
+          <t>H2H Over% (L5)</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>L5 vs Opp Hit%</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>Days Rest</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>Game Total</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>Spread</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Playoff Game</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>Game Script Mult</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>Game Script Note</t>
         </is>
@@ -17121,12 +17819,19 @@
       <c r="BC2" s="3" t="inlineStr"/>
       <c r="BD2" s="3" t="inlineStr"/>
       <c r="BE2" s="3" t="inlineStr"/>
-      <c r="BF2" s="3" t="inlineStr">
+      <c r="BF2" s="3" t="inlineStr"/>
+      <c r="BG2" s="3" t="inlineStr"/>
+      <c r="BH2" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI2" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG2" s="3" t="inlineStr">
+      <c r="BJ2" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -17336,12 +18041,19 @@
       <c r="BC3" s="5" t="inlineStr"/>
       <c r="BD3" s="5" t="inlineStr"/>
       <c r="BE3" s="5" t="inlineStr"/>
-      <c r="BF3" s="5" t="inlineStr">
+      <c r="BF3" s="5" t="inlineStr"/>
+      <c r="BG3" s="5" t="inlineStr"/>
+      <c r="BH3" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI3" s="5" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG3" s="5" t="inlineStr">
+      <c r="BJ3" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -17535,12 +18247,19 @@
       <c r="BC4" s="3" t="inlineStr"/>
       <c r="BD4" s="3" t="inlineStr"/>
       <c r="BE4" s="3" t="inlineStr"/>
-      <c r="BF4" s="3" t="inlineStr">
+      <c r="BF4" s="3" t="inlineStr"/>
+      <c r="BG4" s="3" t="inlineStr"/>
+      <c r="BH4" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI4" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG4" s="3" t="inlineStr">
+      <c r="BJ4" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -17734,12 +18453,19 @@
       <c r="BC5" s="5" t="inlineStr"/>
       <c r="BD5" s="5" t="inlineStr"/>
       <c r="BE5" s="5" t="inlineStr"/>
-      <c r="BF5" s="5" t="inlineStr">
+      <c r="BF5" s="5" t="inlineStr"/>
+      <c r="BG5" s="5" t="inlineStr"/>
+      <c r="BH5" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI5" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG5" s="5" t="inlineStr">
+      <c r="BJ5" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -17945,12 +18671,19 @@
       <c r="BC6" s="3" t="inlineStr"/>
       <c r="BD6" s="3" t="inlineStr"/>
       <c r="BE6" s="3" t="inlineStr"/>
-      <c r="BF6" s="3" t="inlineStr">
+      <c r="BF6" s="3" t="inlineStr"/>
+      <c r="BG6" s="3" t="inlineStr"/>
+      <c r="BH6" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI6" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG6" s="3" t="inlineStr">
+      <c r="BJ6" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -18160,12 +18893,19 @@
       <c r="BC7" s="5" t="inlineStr"/>
       <c r="BD7" s="5" t="inlineStr"/>
       <c r="BE7" s="5" t="inlineStr"/>
-      <c r="BF7" s="5" t="inlineStr">
+      <c r="BF7" s="5" t="inlineStr"/>
+      <c r="BG7" s="5" t="inlineStr"/>
+      <c r="BH7" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI7" s="5" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG7" s="5" t="inlineStr">
+      <c r="BJ7" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -18375,12 +19115,19 @@
       <c r="BC8" s="3" t="inlineStr"/>
       <c r="BD8" s="3" t="inlineStr"/>
       <c r="BE8" s="3" t="inlineStr"/>
-      <c r="BF8" s="3" t="inlineStr">
+      <c r="BF8" s="3" t="inlineStr"/>
+      <c r="BG8" s="3" t="inlineStr"/>
+      <c r="BH8" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI8" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG8" s="3" t="inlineStr">
+      <c r="BJ8" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -18578,12 +19325,19 @@
       <c r="BC9" s="5" t="inlineStr"/>
       <c r="BD9" s="5" t="inlineStr"/>
       <c r="BE9" s="5" t="inlineStr"/>
-      <c r="BF9" s="5" t="inlineStr">
+      <c r="BF9" s="5" t="inlineStr"/>
+      <c r="BG9" s="5" t="inlineStr"/>
+      <c r="BH9" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI9" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG9" s="5" t="inlineStr">
+      <c r="BJ9" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -18793,12 +19547,19 @@
       <c r="BC10" s="3" t="inlineStr"/>
       <c r="BD10" s="3" t="inlineStr"/>
       <c r="BE10" s="3" t="inlineStr"/>
-      <c r="BF10" s="3" t="inlineStr">
+      <c r="BF10" s="3" t="inlineStr"/>
+      <c r="BG10" s="3" t="inlineStr"/>
+      <c r="BH10" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI10" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG10" s="3" t="inlineStr">
+      <c r="BJ10" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -18976,19 +19737,26 @@
       <c r="BC11" s="5" t="inlineStr"/>
       <c r="BD11" s="5" t="inlineStr"/>
       <c r="BE11" s="5" t="inlineStr"/>
-      <c r="BF11" s="5" t="inlineStr">
+      <c r="BF11" s="5" t="inlineStr"/>
+      <c r="BG11" s="5" t="inlineStr"/>
+      <c r="BH11" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI11" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG11" s="5" t="inlineStr">
+      <c r="BJ11" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BG1"/>
+  <autoFilter ref="A1:BJ1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18999,7 +19767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG77"/>
+  <dimension ref="A1:BJ77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -19061,6 +19829,9 @@
     <col width="12" customWidth="1" min="57" max="57"/>
     <col width="12" customWidth="1" min="58" max="58"/>
     <col width="12" customWidth="1" min="59" max="59"/>
+    <col width="12" customWidth="1" min="60" max="60"/>
+    <col width="12" customWidth="1" min="61" max="61"/>
+    <col width="12" customWidth="1" min="62" max="62"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -19331,30 +20102,45 @@
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
+          <t>H2H Over% (L5)</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>L5 vs Opp Hit%</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>Days Rest</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>Game Total</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>Spread</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Playoff Game</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>Game Script Mult</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>Game Script Note</t>
         </is>
@@ -19556,12 +20342,19 @@
       <c r="BC2" s="3" t="inlineStr"/>
       <c r="BD2" s="3" t="inlineStr"/>
       <c r="BE2" s="3" t="inlineStr"/>
-      <c r="BF2" s="3" t="inlineStr">
+      <c r="BF2" s="3" t="inlineStr"/>
+      <c r="BG2" s="3" t="inlineStr"/>
+      <c r="BH2" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI2" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG2" s="3" t="inlineStr">
+      <c r="BJ2" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -19767,12 +20560,19 @@
       <c r="BC3" s="5" t="inlineStr"/>
       <c r="BD3" s="5" t="inlineStr"/>
       <c r="BE3" s="5" t="inlineStr"/>
-      <c r="BF3" s="5" t="inlineStr">
+      <c r="BF3" s="5" t="inlineStr"/>
+      <c r="BG3" s="5" t="inlineStr"/>
+      <c r="BH3" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI3" s="5" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG3" s="5" t="inlineStr">
+      <c r="BJ3" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -19982,12 +20782,19 @@
       <c r="BC4" s="3" t="inlineStr"/>
       <c r="BD4" s="3" t="inlineStr"/>
       <c r="BE4" s="3" t="inlineStr"/>
-      <c r="BF4" s="3" t="inlineStr">
+      <c r="BF4" s="3" t="inlineStr"/>
+      <c r="BG4" s="3" t="inlineStr"/>
+      <c r="BH4" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI4" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG4" s="3" t="inlineStr">
+      <c r="BJ4" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -20193,12 +21000,19 @@
       <c r="BC5" s="5" t="inlineStr"/>
       <c r="BD5" s="5" t="inlineStr"/>
       <c r="BE5" s="5" t="inlineStr"/>
-      <c r="BF5" s="5" t="inlineStr">
+      <c r="BF5" s="5" t="inlineStr"/>
+      <c r="BG5" s="5" t="inlineStr"/>
+      <c r="BH5" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI5" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG5" s="5" t="inlineStr">
+      <c r="BJ5" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -20388,12 +21202,19 @@
       <c r="BC6" s="3" t="inlineStr"/>
       <c r="BD6" s="3" t="inlineStr"/>
       <c r="BE6" s="3" t="inlineStr"/>
-      <c r="BF6" s="3" t="inlineStr">
+      <c r="BF6" s="3" t="inlineStr"/>
+      <c r="BG6" s="3" t="inlineStr"/>
+      <c r="BH6" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI6" s="3" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG6" s="3" t="inlineStr">
+      <c r="BJ6" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -20603,12 +21424,19 @@
       <c r="BC7" s="5" t="inlineStr"/>
       <c r="BD7" s="5" t="inlineStr"/>
       <c r="BE7" s="5" t="inlineStr"/>
-      <c r="BF7" s="5" t="inlineStr">
+      <c r="BF7" s="5" t="inlineStr"/>
+      <c r="BG7" s="5" t="inlineStr"/>
+      <c r="BH7" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI7" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG7" s="5" t="inlineStr">
+      <c r="BJ7" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -20818,12 +21646,19 @@
       <c r="BC8" s="3" t="inlineStr"/>
       <c r="BD8" s="3" t="inlineStr"/>
       <c r="BE8" s="3" t="inlineStr"/>
-      <c r="BF8" s="3" t="inlineStr">
+      <c r="BF8" s="3" t="inlineStr"/>
+      <c r="BG8" s="3" t="inlineStr"/>
+      <c r="BH8" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI8" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG8" s="3" t="inlineStr">
+      <c r="BJ8" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -21029,12 +21864,19 @@
       <c r="BC9" s="5" t="inlineStr"/>
       <c r="BD9" s="5" t="inlineStr"/>
       <c r="BE9" s="5" t="inlineStr"/>
-      <c r="BF9" s="5" t="inlineStr">
+      <c r="BF9" s="5" t="inlineStr"/>
+      <c r="BG9" s="5" t="inlineStr"/>
+      <c r="BH9" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI9" s="5" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG9" s="5" t="inlineStr">
+      <c r="BJ9" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -21236,12 +22078,19 @@
       <c r="BC10" s="3" t="inlineStr"/>
       <c r="BD10" s="3" t="inlineStr"/>
       <c r="BE10" s="3" t="inlineStr"/>
-      <c r="BF10" s="3" t="inlineStr">
+      <c r="BF10" s="3" t="inlineStr"/>
+      <c r="BG10" s="3" t="inlineStr"/>
+      <c r="BH10" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI10" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG10" s="3" t="inlineStr">
+      <c r="BJ10" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -21447,12 +22296,19 @@
       <c r="BC11" s="5" t="inlineStr"/>
       <c r="BD11" s="5" t="inlineStr"/>
       <c r="BE11" s="5" t="inlineStr"/>
-      <c r="BF11" s="5" t="inlineStr">
+      <c r="BF11" s="5" t="inlineStr"/>
+      <c r="BG11" s="5" t="inlineStr"/>
+      <c r="BH11" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI11" s="5" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG11" s="5" t="inlineStr">
+      <c r="BJ11" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -21654,12 +22510,19 @@
       <c r="BC12" s="3" t="inlineStr"/>
       <c r="BD12" s="3" t="inlineStr"/>
       <c r="BE12" s="3" t="inlineStr"/>
-      <c r="BF12" s="3" t="inlineStr">
+      <c r="BF12" s="3" t="inlineStr"/>
+      <c r="BG12" s="3" t="inlineStr"/>
+      <c r="BH12" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI12" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG12" s="3" t="inlineStr">
+      <c r="BJ12" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -21849,12 +22712,19 @@
       <c r="BC13" s="5" t="inlineStr"/>
       <c r="BD13" s="5" t="inlineStr"/>
       <c r="BE13" s="5" t="inlineStr"/>
-      <c r="BF13" s="5" t="inlineStr">
+      <c r="BF13" s="5" t="inlineStr"/>
+      <c r="BG13" s="5" t="inlineStr"/>
+      <c r="BH13" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI13" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG13" s="5" t="inlineStr">
+      <c r="BJ13" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -22064,12 +22934,19 @@
       <c r="BC14" s="3" t="inlineStr"/>
       <c r="BD14" s="3" t="inlineStr"/>
       <c r="BE14" s="3" t="inlineStr"/>
-      <c r="BF14" s="3" t="inlineStr">
+      <c r="BF14" s="3" t="inlineStr"/>
+      <c r="BG14" s="3" t="inlineStr"/>
+      <c r="BH14" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI14" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG14" s="3" t="inlineStr">
+      <c r="BJ14" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -22279,12 +23156,19 @@
       <c r="BC15" s="5" t="inlineStr"/>
       <c r="BD15" s="5" t="inlineStr"/>
       <c r="BE15" s="5" t="inlineStr"/>
-      <c r="BF15" s="5" t="inlineStr">
+      <c r="BF15" s="5" t="inlineStr"/>
+      <c r="BG15" s="5" t="inlineStr"/>
+      <c r="BH15" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI15" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG15" s="5" t="inlineStr">
+      <c r="BJ15" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -22490,12 +23374,19 @@
       <c r="BC16" s="3" t="inlineStr"/>
       <c r="BD16" s="3" t="inlineStr"/>
       <c r="BE16" s="3" t="inlineStr"/>
-      <c r="BF16" s="3" t="inlineStr">
+      <c r="BF16" s="3" t="inlineStr"/>
+      <c r="BG16" s="3" t="inlineStr"/>
+      <c r="BH16" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI16" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG16" s="3" t="inlineStr">
+      <c r="BJ16" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -22701,12 +23592,19 @@
       <c r="BC17" s="5" t="inlineStr"/>
       <c r="BD17" s="5" t="inlineStr"/>
       <c r="BE17" s="5" t="inlineStr"/>
-      <c r="BF17" s="5" t="inlineStr">
+      <c r="BF17" s="5" t="inlineStr"/>
+      <c r="BG17" s="5" t="inlineStr"/>
+      <c r="BH17" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI17" s="5" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG17" s="5" t="inlineStr">
+      <c r="BJ17" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -22916,12 +23814,19 @@
       <c r="BC18" s="3" t="inlineStr"/>
       <c r="BD18" s="3" t="inlineStr"/>
       <c r="BE18" s="3" t="inlineStr"/>
-      <c r="BF18" s="3" t="inlineStr">
+      <c r="BF18" s="3" t="inlineStr"/>
+      <c r="BG18" s="3" t="inlineStr"/>
+      <c r="BH18" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI18" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG18" s="3" t="inlineStr">
+      <c r="BJ18" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -23127,12 +24032,19 @@
       <c r="BC19" s="5" t="inlineStr"/>
       <c r="BD19" s="5" t="inlineStr"/>
       <c r="BE19" s="5" t="inlineStr"/>
-      <c r="BF19" s="5" t="inlineStr">
+      <c r="BF19" s="5" t="inlineStr"/>
+      <c r="BG19" s="5" t="inlineStr"/>
+      <c r="BH19" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI19" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG19" s="5" t="inlineStr">
+      <c r="BJ19" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -23334,12 +24246,19 @@
       <c r="BC20" s="3" t="inlineStr"/>
       <c r="BD20" s="3" t="inlineStr"/>
       <c r="BE20" s="3" t="inlineStr"/>
-      <c r="BF20" s="3" t="inlineStr">
+      <c r="BF20" s="3" t="inlineStr"/>
+      <c r="BG20" s="3" t="inlineStr"/>
+      <c r="BH20" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI20" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG20" s="3" t="inlineStr">
+      <c r="BJ20" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -23471,12 +24390,19 @@
       <c r="BC21" s="5" t="inlineStr"/>
       <c r="BD21" s="5" t="inlineStr"/>
       <c r="BE21" s="5" t="inlineStr"/>
-      <c r="BF21" s="5" t="inlineStr">
+      <c r="BF21" s="5" t="inlineStr"/>
+      <c r="BG21" s="5" t="inlineStr"/>
+      <c r="BH21" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI21" s="5" t="inlineStr">
         <is>
           <t>1.016</t>
         </is>
       </c>
-      <c r="BG21" s="5" t="inlineStr">
+      <c r="BJ21" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, 3ptmade: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -23608,12 +24534,19 @@
       <c r="BC22" s="3" t="inlineStr"/>
       <c r="BD22" s="3" t="inlineStr"/>
       <c r="BE22" s="3" t="inlineStr"/>
-      <c r="BF22" s="3" t="inlineStr">
+      <c r="BF22" s="3" t="inlineStr"/>
+      <c r="BG22" s="3" t="inlineStr"/>
+      <c r="BH22" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI22" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG22" s="3" t="inlineStr">
+      <c r="BJ22" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -23745,12 +24678,19 @@
       <c r="BC23" s="5" t="inlineStr"/>
       <c r="BD23" s="5" t="inlineStr"/>
       <c r="BE23" s="5" t="inlineStr"/>
-      <c r="BF23" s="5" t="inlineStr">
+      <c r="BF23" s="5" t="inlineStr"/>
+      <c r="BG23" s="5" t="inlineStr"/>
+      <c r="BH23" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI23" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG23" s="5" t="inlineStr">
+      <c r="BJ23" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -23882,12 +24822,19 @@
       <c r="BC24" s="3" t="inlineStr"/>
       <c r="BD24" s="3" t="inlineStr"/>
       <c r="BE24" s="3" t="inlineStr"/>
-      <c r="BF24" s="3" t="inlineStr">
+      <c r="BF24" s="3" t="inlineStr"/>
+      <c r="BG24" s="3" t="inlineStr"/>
+      <c r="BH24" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI24" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG24" s="3" t="inlineStr">
+      <c r="BJ24" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -24019,12 +24966,19 @@
       <c r="BC25" s="5" t="inlineStr"/>
       <c r="BD25" s="5" t="inlineStr"/>
       <c r="BE25" s="5" t="inlineStr"/>
-      <c r="BF25" s="5" t="inlineStr">
+      <c r="BF25" s="5" t="inlineStr"/>
+      <c r="BG25" s="5" t="inlineStr"/>
+      <c r="BH25" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI25" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG25" s="5" t="inlineStr">
+      <c r="BJ25" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -24156,12 +25110,19 @@
       <c r="BC26" s="3" t="inlineStr"/>
       <c r="BD26" s="3" t="inlineStr"/>
       <c r="BE26" s="3" t="inlineStr"/>
-      <c r="BF26" s="3" t="inlineStr">
+      <c r="BF26" s="3" t="inlineStr"/>
+      <c r="BG26" s="3" t="inlineStr"/>
+      <c r="BH26" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI26" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG26" s="3" t="inlineStr">
+      <c r="BJ26" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -24293,12 +25254,19 @@
       <c r="BC27" s="5" t="inlineStr"/>
       <c r="BD27" s="5" t="inlineStr"/>
       <c r="BE27" s="5" t="inlineStr"/>
-      <c r="BF27" s="5" t="inlineStr">
+      <c r="BF27" s="5" t="inlineStr"/>
+      <c r="BG27" s="5" t="inlineStr"/>
+      <c r="BH27" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI27" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG27" s="5" t="inlineStr">
+      <c r="BJ27" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -24430,12 +25398,19 @@
       <c r="BC28" s="3" t="inlineStr"/>
       <c r="BD28" s="3" t="inlineStr"/>
       <c r="BE28" s="3" t="inlineStr"/>
-      <c r="BF28" s="3" t="inlineStr">
+      <c r="BF28" s="3" t="inlineStr"/>
+      <c r="BG28" s="3" t="inlineStr"/>
+      <c r="BH28" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI28" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG28" s="3" t="inlineStr">
+      <c r="BJ28" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -24567,12 +25542,19 @@
       <c r="BC29" s="5" t="inlineStr"/>
       <c r="BD29" s="5" t="inlineStr"/>
       <c r="BE29" s="5" t="inlineStr"/>
-      <c r="BF29" s="5" t="inlineStr">
+      <c r="BF29" s="5" t="inlineStr"/>
+      <c r="BG29" s="5" t="inlineStr"/>
+      <c r="BH29" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI29" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG29" s="5" t="inlineStr">
+      <c r="BJ29" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -24704,12 +25686,19 @@
       <c r="BC30" s="3" t="inlineStr"/>
       <c r="BD30" s="3" t="inlineStr"/>
       <c r="BE30" s="3" t="inlineStr"/>
-      <c r="BF30" s="3" t="inlineStr">
+      <c r="BF30" s="3" t="inlineStr"/>
+      <c r="BG30" s="3" t="inlineStr"/>
+      <c r="BH30" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI30" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG30" s="3" t="inlineStr">
+      <c r="BJ30" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -24841,12 +25830,19 @@
       <c r="BC31" s="5" t="inlineStr"/>
       <c r="BD31" s="5" t="inlineStr"/>
       <c r="BE31" s="5" t="inlineStr"/>
-      <c r="BF31" s="5" t="inlineStr">
+      <c r="BF31" s="5" t="inlineStr"/>
+      <c r="BG31" s="5" t="inlineStr"/>
+      <c r="BH31" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI31" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG31" s="5" t="inlineStr">
+      <c r="BJ31" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -25038,12 +26034,19 @@
       <c r="BC32" s="3" t="inlineStr"/>
       <c r="BD32" s="3" t="inlineStr"/>
       <c r="BE32" s="3" t="inlineStr"/>
-      <c r="BF32" s="3" t="inlineStr">
+      <c r="BF32" s="3" t="inlineStr"/>
+      <c r="BG32" s="3" t="inlineStr"/>
+      <c r="BH32" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI32" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG32" s="3" t="inlineStr">
+      <c r="BJ32" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -25175,12 +26178,19 @@
       <c r="BC33" s="5" t="inlineStr"/>
       <c r="BD33" s="5" t="inlineStr"/>
       <c r="BE33" s="5" t="inlineStr"/>
-      <c r="BF33" s="5" t="inlineStr">
+      <c r="BF33" s="5" t="inlineStr"/>
+      <c r="BG33" s="5" t="inlineStr"/>
+      <c r="BH33" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI33" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG33" s="5" t="inlineStr">
+      <c r="BJ33" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -25388,12 +26398,19 @@
       <c r="BC34" s="3" t="inlineStr"/>
       <c r="BD34" s="3" t="inlineStr"/>
       <c r="BE34" s="3" t="inlineStr"/>
-      <c r="BF34" s="3" t="inlineStr">
+      <c r="BF34" s="3" t="inlineStr"/>
+      <c r="BG34" s="3" t="inlineStr"/>
+      <c r="BH34" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI34" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG34" s="3" t="inlineStr">
+      <c r="BJ34" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -25525,12 +26542,19 @@
       <c r="BC35" s="5" t="inlineStr"/>
       <c r="BD35" s="5" t="inlineStr"/>
       <c r="BE35" s="5" t="inlineStr"/>
-      <c r="BF35" s="5" t="inlineStr">
+      <c r="BF35" s="5" t="inlineStr"/>
+      <c r="BG35" s="5" t="inlineStr"/>
+      <c r="BH35" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI35" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG35" s="5" t="inlineStr">
+      <c r="BJ35" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -25662,12 +26686,19 @@
       <c r="BC36" s="3" t="inlineStr"/>
       <c r="BD36" s="3" t="inlineStr"/>
       <c r="BE36" s="3" t="inlineStr"/>
-      <c r="BF36" s="3" t="inlineStr">
+      <c r="BF36" s="3" t="inlineStr"/>
+      <c r="BG36" s="3" t="inlineStr"/>
+      <c r="BH36" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI36" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG36" s="3" t="inlineStr">
+      <c r="BJ36" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -25863,12 +26894,19 @@
       <c r="BC37" s="5" t="inlineStr"/>
       <c r="BD37" s="5" t="inlineStr"/>
       <c r="BE37" s="5" t="inlineStr"/>
-      <c r="BF37" s="5" t="inlineStr">
+      <c r="BF37" s="5" t="inlineStr"/>
+      <c r="BG37" s="5" t="inlineStr"/>
+      <c r="BH37" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI37" s="5" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG37" s="5" t="inlineStr">
+      <c r="BJ37" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -26000,12 +27038,19 @@
       <c r="BC38" s="3" t="inlineStr"/>
       <c r="BD38" s="3" t="inlineStr"/>
       <c r="BE38" s="3" t="inlineStr"/>
-      <c r="BF38" s="3" t="inlineStr">
+      <c r="BF38" s="3" t="inlineStr"/>
+      <c r="BG38" s="3" t="inlineStr"/>
+      <c r="BH38" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI38" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG38" s="3" t="inlineStr">
+      <c r="BJ38" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -26137,12 +27182,19 @@
       <c r="BC39" s="5" t="inlineStr"/>
       <c r="BD39" s="5" t="inlineStr"/>
       <c r="BE39" s="5" t="inlineStr"/>
-      <c r="BF39" s="5" t="inlineStr">
+      <c r="BF39" s="5" t="inlineStr"/>
+      <c r="BG39" s="5" t="inlineStr"/>
+      <c r="BH39" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI39" s="5" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="BG39" s="5" t="inlineStr">
+      <c r="BJ39" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, pts: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -26274,12 +27326,19 @@
       <c r="BC40" s="3" t="inlineStr"/>
       <c r="BD40" s="3" t="inlineStr"/>
       <c r="BE40" s="3" t="inlineStr"/>
-      <c r="BF40" s="3" t="inlineStr">
+      <c r="BF40" s="3" t="inlineStr"/>
+      <c r="BG40" s="3" t="inlineStr"/>
+      <c r="BH40" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI40" s="3" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG40" s="3" t="inlineStr">
+      <c r="BJ40" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -26411,12 +27470,19 @@
       <c r="BC41" s="5" t="inlineStr"/>
       <c r="BD41" s="5" t="inlineStr"/>
       <c r="BE41" s="5" t="inlineStr"/>
-      <c r="BF41" s="5" t="inlineStr">
+      <c r="BF41" s="5" t="inlineStr"/>
+      <c r="BG41" s="5" t="inlineStr"/>
+      <c r="BH41" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI41" s="5" t="inlineStr">
         <is>
           <t>1.016</t>
         </is>
       </c>
-      <c r="BG41" s="5" t="inlineStr">
+      <c r="BJ41" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, 3ptmade: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -26548,12 +27614,19 @@
       <c r="BC42" s="3" t="inlineStr"/>
       <c r="BD42" s="3" t="inlineStr"/>
       <c r="BE42" s="3" t="inlineStr"/>
-      <c r="BF42" s="3" t="inlineStr">
+      <c r="BF42" s="3" t="inlineStr"/>
+      <c r="BG42" s="3" t="inlineStr"/>
+      <c r="BH42" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI42" s="3" t="inlineStr">
         <is>
           <t>1.016</t>
         </is>
       </c>
-      <c r="BG42" s="3" t="inlineStr">
+      <c r="BJ42" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, 3ptmade: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -26685,12 +27758,19 @@
       <c r="BC43" s="5" t="inlineStr"/>
       <c r="BD43" s="5" t="inlineStr"/>
       <c r="BE43" s="5" t="inlineStr"/>
-      <c r="BF43" s="5" t="inlineStr">
+      <c r="BF43" s="5" t="inlineStr"/>
+      <c r="BG43" s="5" t="inlineStr"/>
+      <c r="BH43" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI43" s="5" t="inlineStr">
         <is>
           <t>1.016</t>
         </is>
       </c>
-      <c r="BG43" s="5" t="inlineStr">
+      <c r="BJ43" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, 3ptmade: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -26822,12 +27902,19 @@
       <c r="BC44" s="3" t="inlineStr"/>
       <c r="BD44" s="3" t="inlineStr"/>
       <c r="BE44" s="3" t="inlineStr"/>
-      <c r="BF44" s="3" t="inlineStr">
+      <c r="BF44" s="3" t="inlineStr"/>
+      <c r="BG44" s="3" t="inlineStr"/>
+      <c r="BH44" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI44" s="3" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG44" s="3" t="inlineStr">
+      <c r="BJ44" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -26959,12 +28046,19 @@
       <c r="BC45" s="5" t="inlineStr"/>
       <c r="BD45" s="5" t="inlineStr"/>
       <c r="BE45" s="5" t="inlineStr"/>
-      <c r="BF45" s="5" t="inlineStr">
+      <c r="BF45" s="5" t="inlineStr"/>
+      <c r="BG45" s="5" t="inlineStr"/>
+      <c r="BH45" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI45" s="5" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG45" s="5" t="inlineStr">
+      <c r="BJ45" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -27096,12 +28190,19 @@
       <c r="BC46" s="3" t="inlineStr"/>
       <c r="BD46" s="3" t="inlineStr"/>
       <c r="BE46" s="3" t="inlineStr"/>
-      <c r="BF46" s="3" t="inlineStr">
+      <c r="BF46" s="3" t="inlineStr"/>
+      <c r="BG46" s="3" t="inlineStr"/>
+      <c r="BH46" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI46" s="3" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG46" s="3" t="inlineStr">
+      <c r="BJ46" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -27233,12 +28334,19 @@
       <c r="BC47" s="5" t="inlineStr"/>
       <c r="BD47" s="5" t="inlineStr"/>
       <c r="BE47" s="5" t="inlineStr"/>
-      <c r="BF47" s="5" t="inlineStr">
+      <c r="BF47" s="5" t="inlineStr"/>
+      <c r="BG47" s="5" t="inlineStr"/>
+      <c r="BH47" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI47" s="5" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG47" s="5" t="inlineStr">
+      <c r="BJ47" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -27370,12 +28478,19 @@
       <c r="BC48" s="3" t="inlineStr"/>
       <c r="BD48" s="3" t="inlineStr"/>
       <c r="BE48" s="3" t="inlineStr"/>
-      <c r="BF48" s="3" t="inlineStr">
+      <c r="BF48" s="3" t="inlineStr"/>
+      <c r="BG48" s="3" t="inlineStr"/>
+      <c r="BH48" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI48" s="3" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG48" s="3" t="inlineStr">
+      <c r="BJ48" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -27507,12 +28622,19 @@
       <c r="BC49" s="5" t="inlineStr"/>
       <c r="BD49" s="5" t="inlineStr"/>
       <c r="BE49" s="5" t="inlineStr"/>
-      <c r="BF49" s="5" t="inlineStr">
+      <c r="BF49" s="5" t="inlineStr"/>
+      <c r="BG49" s="5" t="inlineStr"/>
+      <c r="BH49" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI49" s="5" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG49" s="5" t="inlineStr">
+      <c r="BJ49" s="5" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -27644,12 +28766,19 @@
       <c r="BC50" s="3" t="inlineStr"/>
       <c r="BD50" s="3" t="inlineStr"/>
       <c r="BE50" s="3" t="inlineStr"/>
-      <c r="BF50" s="3" t="inlineStr">
+      <c r="BF50" s="3" t="inlineStr"/>
+      <c r="BG50" s="3" t="inlineStr"/>
+      <c r="BH50" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI50" s="3" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG50" s="3" t="inlineStr">
+      <c r="BJ50" s="3" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -27781,12 +28910,19 @@
       <c r="BC51" s="5" t="inlineStr"/>
       <c r="BD51" s="5" t="inlineStr"/>
       <c r="BE51" s="5" t="inlineStr"/>
-      <c r="BF51" s="5" t="inlineStr">
+      <c r="BF51" s="5" t="inlineStr"/>
+      <c r="BG51" s="5" t="inlineStr"/>
+      <c r="BH51" s="5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI51" s="5" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG51" s="5" t="inlineStr">
+      <c r="BJ51" s="5" t="inlineStr">
         <is>
           <t>CHA +3.5 pt margin vs ORL, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -27918,12 +29054,19 @@
       <c r="BC52" s="3" t="inlineStr"/>
       <c r="BD52" s="3" t="inlineStr"/>
       <c r="BE52" s="3" t="inlineStr"/>
-      <c r="BF52" s="3" t="inlineStr">
+      <c r="BF52" s="3" t="inlineStr"/>
+      <c r="BG52" s="3" t="inlineStr"/>
+      <c r="BH52" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="BI52" s="3" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG52" s="3" t="inlineStr">
+      <c r="BJ52" s="3" t="inlineStr">
         <is>
           <t>ORL -3.5 pt margin vs CHA, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -28055,12 +29198,19 @@
       <c r="BC53" s="5" t="inlineStr"/>
       <c r="BD53" s="5" t="inlineStr"/>
       <c r="BE53" s="5" t="inlineStr"/>
-      <c r="BF53" s="5" t="inlineStr">
+      <c r="BF53" s="5" t="inlineStr"/>
+      <c r="BG53" s="5" t="inlineStr"/>
+      <c r="BH53" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI53" s="5" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG53" s="5" t="inlineStr">
+      <c r="BJ53" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -28192,12 +29342,19 @@
       <c r="BC54" s="3" t="inlineStr"/>
       <c r="BD54" s="3" t="inlineStr"/>
       <c r="BE54" s="3" t="inlineStr"/>
-      <c r="BF54" s="3" t="inlineStr">
+      <c r="BF54" s="3" t="inlineStr"/>
+      <c r="BG54" s="3" t="inlineStr"/>
+      <c r="BH54" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI54" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG54" s="3" t="inlineStr">
+      <c r="BJ54" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -28329,12 +29486,19 @@
       <c r="BC55" s="5" t="inlineStr"/>
       <c r="BD55" s="5" t="inlineStr"/>
       <c r="BE55" s="5" t="inlineStr"/>
-      <c r="BF55" s="5" t="inlineStr">
+      <c r="BF55" s="5" t="inlineStr"/>
+      <c r="BG55" s="5" t="inlineStr"/>
+      <c r="BH55" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI55" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG55" s="5" t="inlineStr">
+      <c r="BJ55" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -28466,12 +29630,19 @@
       <c r="BC56" s="3" t="inlineStr"/>
       <c r="BD56" s="3" t="inlineStr"/>
       <c r="BE56" s="3" t="inlineStr"/>
-      <c r="BF56" s="3" t="inlineStr">
+      <c r="BF56" s="3" t="inlineStr"/>
+      <c r="BG56" s="3" t="inlineStr"/>
+      <c r="BH56" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI56" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG56" s="3" t="inlineStr">
+      <c r="BJ56" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -28603,12 +29774,19 @@
       <c r="BC57" s="5" t="inlineStr"/>
       <c r="BD57" s="5" t="inlineStr"/>
       <c r="BE57" s="5" t="inlineStr"/>
-      <c r="BF57" s="5" t="inlineStr">
+      <c r="BF57" s="5" t="inlineStr"/>
+      <c r="BG57" s="5" t="inlineStr"/>
+      <c r="BH57" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI57" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG57" s="5" t="inlineStr">
+      <c r="BJ57" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -28740,12 +29918,19 @@
       <c r="BC58" s="3" t="inlineStr"/>
       <c r="BD58" s="3" t="inlineStr"/>
       <c r="BE58" s="3" t="inlineStr"/>
-      <c r="BF58" s="3" t="inlineStr">
+      <c r="BF58" s="3" t="inlineStr"/>
+      <c r="BG58" s="3" t="inlineStr"/>
+      <c r="BH58" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI58" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG58" s="3" t="inlineStr">
+      <c r="BJ58" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -28877,12 +30062,19 @@
       <c r="BC59" s="5" t="inlineStr"/>
       <c r="BD59" s="5" t="inlineStr"/>
       <c r="BE59" s="5" t="inlineStr"/>
-      <c r="BF59" s="5" t="inlineStr">
+      <c r="BF59" s="5" t="inlineStr"/>
+      <c r="BG59" s="5" t="inlineStr"/>
+      <c r="BH59" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI59" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG59" s="5" t="inlineStr">
+      <c r="BJ59" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -29014,12 +30206,19 @@
       <c r="BC60" s="3" t="inlineStr"/>
       <c r="BD60" s="3" t="inlineStr"/>
       <c r="BE60" s="3" t="inlineStr"/>
-      <c r="BF60" s="3" t="inlineStr">
+      <c r="BF60" s="3" t="inlineStr"/>
+      <c r="BG60" s="3" t="inlineStr"/>
+      <c r="BH60" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI60" s="3" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG60" s="3" t="inlineStr">
+      <c r="BJ60" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pra: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -29151,12 +30350,19 @@
       <c r="BC61" s="5" t="inlineStr"/>
       <c r="BD61" s="5" t="inlineStr"/>
       <c r="BE61" s="5" t="inlineStr"/>
-      <c r="BF61" s="5" t="inlineStr">
+      <c r="BF61" s="5" t="inlineStr"/>
+      <c r="BG61" s="5" t="inlineStr"/>
+      <c r="BH61" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI61" s="5" t="inlineStr">
         <is>
           <t>0.937</t>
         </is>
       </c>
-      <c r="BG61" s="5" t="inlineStr">
+      <c r="BJ61" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, fantasy: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -29288,12 +30494,19 @@
       <c r="BC62" s="3" t="inlineStr"/>
       <c r="BD62" s="3" t="inlineStr"/>
       <c r="BE62" s="3" t="inlineStr"/>
-      <c r="BF62" s="3" t="inlineStr">
+      <c r="BF62" s="3" t="inlineStr"/>
+      <c r="BG62" s="3" t="inlineStr"/>
+      <c r="BH62" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI62" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG62" s="3" t="inlineStr">
+      <c r="BJ62" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -29425,12 +30638,19 @@
       <c r="BC63" s="5" t="inlineStr"/>
       <c r="BD63" s="5" t="inlineStr"/>
       <c r="BE63" s="5" t="inlineStr"/>
-      <c r="BF63" s="5" t="inlineStr">
+      <c r="BF63" s="5" t="inlineStr"/>
+      <c r="BG63" s="5" t="inlineStr"/>
+      <c r="BH63" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI63" s="5" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG63" s="5" t="inlineStr">
+      <c r="BJ63" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -29562,12 +30782,19 @@
       <c r="BC64" s="3" t="inlineStr"/>
       <c r="BD64" s="3" t="inlineStr"/>
       <c r="BE64" s="3" t="inlineStr"/>
-      <c r="BF64" s="3" t="inlineStr">
+      <c r="BF64" s="3" t="inlineStr"/>
+      <c r="BG64" s="3" t="inlineStr"/>
+      <c r="BH64" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI64" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG64" s="3" t="inlineStr">
+      <c r="BJ64" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, fantasy: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -29699,12 +30926,19 @@
       <c r="BC65" s="5" t="inlineStr"/>
       <c r="BD65" s="5" t="inlineStr"/>
       <c r="BE65" s="5" t="inlineStr"/>
-      <c r="BF65" s="5" t="inlineStr">
+      <c r="BF65" s="5" t="inlineStr"/>
+      <c r="BG65" s="5" t="inlineStr"/>
+      <c r="BH65" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI65" s="5" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="BG65" s="5" t="inlineStr">
+      <c r="BJ65" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, pts: 0.93x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -29884,12 +31118,19 @@
       <c r="BC66" s="3" t="inlineStr"/>
       <c r="BD66" s="3" t="inlineStr"/>
       <c r="BE66" s="3" t="inlineStr"/>
-      <c r="BF66" s="3" t="inlineStr">
+      <c r="BF66" s="3" t="inlineStr"/>
+      <c r="BG66" s="3" t="inlineStr"/>
+      <c r="BH66" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI66" s="3" t="inlineStr">
         <is>
           <t>1.018</t>
         </is>
       </c>
-      <c r="BG66" s="3" t="inlineStr">
+      <c r="BJ66" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, pra: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -30021,12 +31262,19 @@
       <c r="BC67" s="5" t="inlineStr"/>
       <c r="BD67" s="5" t="inlineStr"/>
       <c r="BE67" s="5" t="inlineStr"/>
-      <c r="BF67" s="5" t="inlineStr">
+      <c r="BF67" s="5" t="inlineStr"/>
+      <c r="BG67" s="5" t="inlineStr"/>
+      <c r="BH67" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI67" s="5" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG67" s="5" t="inlineStr">
+      <c r="BJ67" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -30158,12 +31406,19 @@
       <c r="BC68" s="3" t="inlineStr"/>
       <c r="BD68" s="3" t="inlineStr"/>
       <c r="BE68" s="3" t="inlineStr"/>
-      <c r="BF68" s="3" t="inlineStr">
+      <c r="BF68" s="3" t="inlineStr"/>
+      <c r="BG68" s="3" t="inlineStr"/>
+      <c r="BH68" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI68" s="3" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG68" s="3" t="inlineStr">
+      <c r="BJ68" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -30295,12 +31550,19 @@
       <c r="BC69" s="5" t="inlineStr"/>
       <c r="BD69" s="5" t="inlineStr"/>
       <c r="BE69" s="5" t="inlineStr"/>
-      <c r="BF69" s="5" t="inlineStr">
+      <c r="BF69" s="5" t="inlineStr"/>
+      <c r="BG69" s="5" t="inlineStr"/>
+      <c r="BH69" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI69" s="5" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG69" s="5" t="inlineStr">
+      <c r="BJ69" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -30432,12 +31694,19 @@
       <c r="BC70" s="3" t="inlineStr"/>
       <c r="BD70" s="3" t="inlineStr"/>
       <c r="BE70" s="3" t="inlineStr"/>
-      <c r="BF70" s="3" t="inlineStr">
+      <c r="BF70" s="3" t="inlineStr"/>
+      <c r="BG70" s="3" t="inlineStr"/>
+      <c r="BH70" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI70" s="3" t="inlineStr">
         <is>
           <t>1.016</t>
         </is>
       </c>
-      <c r="BG70" s="3" t="inlineStr">
+      <c r="BJ70" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, 3ptmade: 1.02x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -30569,12 +31838,19 @@
       <c r="BC71" s="5" t="inlineStr"/>
       <c r="BD71" s="5" t="inlineStr"/>
       <c r="BE71" s="5" t="inlineStr"/>
-      <c r="BF71" s="5" t="inlineStr">
+      <c r="BF71" s="5" t="inlineStr"/>
+      <c r="BG71" s="5" t="inlineStr"/>
+      <c r="BH71" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI71" s="5" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG71" s="5" t="inlineStr">
+      <c r="BJ71" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -30706,12 +31982,19 @@
       <c r="BC72" s="3" t="inlineStr"/>
       <c r="BD72" s="3" t="inlineStr"/>
       <c r="BE72" s="3" t="inlineStr"/>
-      <c r="BF72" s="3" t="inlineStr">
+      <c r="BF72" s="3" t="inlineStr"/>
+      <c r="BG72" s="3" t="inlineStr"/>
+      <c r="BH72" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI72" s="3" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG72" s="3" t="inlineStr">
+      <c r="BJ72" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -30843,12 +32126,19 @@
       <c r="BC73" s="5" t="inlineStr"/>
       <c r="BD73" s="5" t="inlineStr"/>
       <c r="BE73" s="5" t="inlineStr"/>
-      <c r="BF73" s="5" t="inlineStr">
+      <c r="BF73" s="5" t="inlineStr"/>
+      <c r="BG73" s="5" t="inlineStr"/>
+      <c r="BH73" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI73" s="5" t="inlineStr">
         <is>
           <t>0.944</t>
         </is>
       </c>
-      <c r="BG73" s="5" t="inlineStr">
+      <c r="BJ73" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, 3ptmade: 0.94x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -30980,12 +32270,19 @@
       <c r="BC74" s="3" t="inlineStr"/>
       <c r="BD74" s="3" t="inlineStr"/>
       <c r="BE74" s="3" t="inlineStr"/>
-      <c r="BF74" s="3" t="inlineStr">
+      <c r="BF74" s="3" t="inlineStr"/>
+      <c r="BG74" s="3" t="inlineStr"/>
+      <c r="BH74" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI74" s="3" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG74" s="3" t="inlineStr">
+      <c r="BJ74" s="3" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -31117,12 +32414,19 @@
       <c r="BC75" s="5" t="inlineStr"/>
       <c r="BD75" s="5" t="inlineStr"/>
       <c r="BE75" s="5" t="inlineStr"/>
-      <c r="BF75" s="5" t="inlineStr">
+      <c r="BF75" s="5" t="inlineStr"/>
+      <c r="BG75" s="5" t="inlineStr"/>
+      <c r="BH75" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI75" s="5" t="inlineStr">
         <is>
           <t>1.014</t>
         </is>
       </c>
-      <c r="BG75" s="5" t="inlineStr">
+      <c r="BJ75" s="5" t="inlineStr">
         <is>
           <t>PHX +3.5 pt margin vs ?, ftm: 1.01x game script (fav; spread_risk 1.02, total_risk 1.00)</t>
         </is>
@@ -31254,12 +32558,19 @@
       <c r="BC76" s="3" t="inlineStr"/>
       <c r="BD76" s="3" t="inlineStr"/>
       <c r="BE76" s="3" t="inlineStr"/>
-      <c r="BF76" s="3" t="inlineStr">
+      <c r="BF76" s="3" t="inlineStr"/>
+      <c r="BG76" s="3" t="inlineStr"/>
+      <c r="BH76" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI76" s="3" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG76" s="3" t="inlineStr">
+      <c r="BJ76" s="3" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
@@ -31391,19 +32702,26 @@
       <c r="BC77" s="5" t="inlineStr"/>
       <c r="BD77" s="5" t="inlineStr"/>
       <c r="BE77" s="5" t="inlineStr"/>
-      <c r="BF77" s="5" t="inlineStr">
+      <c r="BF77" s="5" t="inlineStr"/>
+      <c r="BG77" s="5" t="inlineStr"/>
+      <c r="BH77" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI77" s="5" t="inlineStr">
         <is>
           <t>0.951</t>
         </is>
       </c>
-      <c r="BG77" s="5" t="inlineStr">
+      <c r="BJ77" s="5" t="inlineStr">
         <is>
           <t>GSW -3.5 pt margin vs ?, ftm: 0.95x game script (dog; spread_risk 0.93, total_risk 1.00)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BG1"/>
+  <autoFilter ref="A1:BJ1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>